<commit_message>
tự động logout khi đổi mật khẩu
</commit_message>
<xml_diff>
--- a/import_file_test/Hoi_Thi_Chuyen_Mon_Thang_8_Z176.xlsx
+++ b/import_file_test/Hoi_Thi_Chuyen_Mon_Thang_8_Z176.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P52"/>
+  <dimension ref="A1:P57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3581,6 +3581,316 @@
         </is>
       </c>
       <c r="P52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Hội thi chuyên môn cho nhân viên tháng 8</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Phòng test chịu trách nhiệm chính về công việc gì trong đơn vị?</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Lý thuyết</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Dễ</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Chọn 1</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Riêng</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Phòng test</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Kiểm thử và đảm bảo chất lượng quy trình/hệ thống nội bộ</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Quản lý nhân sự toàn công ty</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Sản xuất trực tiếp tại xưởng</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Kế toán tổng hợp</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Hội thi chuyên môn cho nhân viên tháng 8</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Khi phát hiện lỗi trong quy trình đang kiểm thử, nhân viên Phòng test cần làm gì đầu tiên?</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Bài tập</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Chọn 1</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Riêng</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Phòng test</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Ghi nhận đầy đủ thông tin lỗi và báo cáo cho bộ phận liên quan</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Tự ý sửa lỗi mà không báo cáo</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Bỏ qua vì không thuộc trách nhiệm</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Xóa toàn bộ dữ liệu kiểm thử</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Hội thi chuyên môn cho nhân viên tháng 8</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Mục tiêu chính của việc kiểm thử trước khi triển khai là gì?</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Lý thuyết</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Dễ</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Chọn 1</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Riêng</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Phòng test</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Phát hiện sớm lỗi để giảm rủi ro khi vận hành thực tế</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Làm chậm tiến độ dự án</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Tăng khối lượng công việc không cần thiết</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Không có mục tiêu rõ ràng</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Hội thi chuyên môn cho nhân viên tháng 8</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Khi lập báo cáo kết quả kiểm thử, nội dung nào sau đây là bắt buộc?</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Bài tập</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Khó</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Chọn nhiều</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Riêng</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Phòng test</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Danh sách lỗi phát hiện được</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Mức độ ảnh hưởng của từng lỗi</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Đề xuất hướng khắc phục</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Thông tin lương thưởng nhân viên</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Hội thi chuyên môn cho nhân viên tháng 8</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Phòng test nên phối hợp với bộ phận nào để xử lý lỗi phát sinh sau kiểm thử?</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Lý thuyết</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Chọn 1</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Riêng</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Phòng test</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Bộ phận phát triển/vận hành hệ thống liên quan</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Bộ phận lễ tân</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Bộ phận bảo vệ</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Không cần phối hợp với ai</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -3729,7 +4039,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>15 câu Chung + 36 câu Riêng (9 bộ phận) = 51 câu tổng. Chủ đề MỚI (chưa tồn tại trong hệ thống) để test tạo Topic tự động.</t>
+          <t>15 câu Chung + 36 câu Riêng (9 bộ phận cũ) + 5 câu Riêng (Phòng test - bộ phận MỚI, 0 nhân viên) = 56 câu tổng. Chủ đề MỚI để test tạo Topic tự động. "Phòng test" dùng để test bug ExamCode khi phòng ban 0 nhân viên tại thời điểm publish.</t>
         </is>
       </c>
     </row>

</xml_diff>